<commit_message>
fix(p1): version normative gate inputs
</commit_message>
<xml_diff>
--- a/products-storage/01-zakrytie-rabot/14-raschet-procentov-395-gk.xlsx
+++ b/products-storage/01-zakrytie-rabot/14-raschet-procentov-395-gk.xlsx
@@ -22,7 +22,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="DD.MM.YYYY"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -57,6 +57,12 @@
     </font>
     <font>
       <name val="Times New Roman"/>
+      <color rgb="00C00000"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Times New Roman"/>
+      <b val="1"/>
       <color rgb="00C00000"/>
       <sz val="10"/>
     </font>
@@ -116,7 +122,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -139,12 +145,13 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="4" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="1" fontId="7" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="8" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="8" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -764,7 +771,7 @@
     <row r="47" ht="64" customHeight="1">
       <c r="A47" s="5" t="inlineStr">
         <is>
-          <t>Частичная оплата по ст. 319 ГК РФ гасит сначала издержки, затем проценты и только потом основной долг. Отступить от этой очерёдности можно соглашением сторон; одностороннее указание в платёжном поручении соглашением не является и очерёдность не меняет. Порядок такой: есть допустимое соглашение — считайте по нему; соглашения нет — по ст. 319 ГК РФ. Если однородных обязательств несколько, выбор погашаемого — отдельный вопрос, и его решают не здесь. Эта таблица уменьшает базу долга на сумму оплаты с её даты, то есть считает по простому варианту: если очерёдность имеет значение для вашего спора, расчёт надо корректировать с юристом.</t>
+          <t>Частичная оплата по ст. 319 ГК РФ гасит сначала издержки, затем проценты и только потом основной долг. Отступить от этой очерёдности можно соглашением сторон; одностороннее указание в платёжном поручении соглашением не является и очерёдность не меняет. Порядок такой: есть допустимое соглашение — считайте по нему; соглашения нет — по ст. 319 ГК РФ. Если однородных обязательств несколько, выбор погашаемого — отдельный вопрос, и его решают не здесь. Эта таблица уменьшает базу долга со дня, следующего за датой оплаты: день оплаты остаётся днём просрочки на прежнюю сумму. Это простой вариант; если очерёдность имеет значение для вашего спора, расчёт надо корректировать с юристом.</t>
         </is>
       </c>
     </row>
@@ -861,7 +868,7 @@
         <v/>
       </c>
       <c r="D4" s="11">
-        <f>IF($A4="","",'Входные данные'!$B$4-SUMIF('Входные данные'!$A$35:$A$44,"&lt;="&amp;$A4,'Входные данные'!$B$35:$B$44))</f>
+        <f>IF($A4="","",'Входные данные'!$B$4-SUMIF('Входные данные'!$A$35:$A$44,"&lt;"&amp;$A4,'Входные данные'!$B$35:$B$44))</f>
         <v/>
       </c>
       <c r="E4" s="12">
@@ -877,7 +884,7 @@
         <v/>
       </c>
       <c r="H4" s="13">
-        <f>IF($A4="","",IF(YEAR($A4)&lt;&gt;YEAR($B4),"Период пересекает 31 декабря — разбейте на две строки",IF($B4&lt;$A4,"Конец периода раньше начала",IF($E4="","Ставка на эту дату не найдена: дополните таблицу ставок",""))))</f>
+        <f>IF($A4="","",IF(YEAR($A4)&lt;&gt;YEAR($B4),"Период пересекает 31 декабря — разбейте на две строки",IF($B4&lt;$A4,"Конец периода раньше начала",IF($A4&lt;&gt;'Входные данные'!$B$5,"Период пропущен или перекрыт — исправьте даты",IF($E4="","Ставка на эту дату не найдена: дополните таблицу ставок","")))))</f>
         <v/>
       </c>
     </row>
@@ -889,7 +896,7 @@
         <v/>
       </c>
       <c r="D5" s="11">
-        <f>IF($A5="","",'Входные данные'!$B$4-SUMIF('Входные данные'!$A$35:$A$44,"&lt;="&amp;$A5,'Входные данные'!$B$35:$B$44))</f>
+        <f>IF($A5="","",'Входные данные'!$B$4-SUMIF('Входные данные'!$A$35:$A$44,"&lt;"&amp;$A5,'Входные данные'!$B$35:$B$44))</f>
         <v/>
       </c>
       <c r="E5" s="12">
@@ -905,7 +912,7 @@
         <v/>
       </c>
       <c r="H5" s="13">
-        <f>IF($A5="","",IF(YEAR($A5)&lt;&gt;YEAR($B5),"Период пересекает 31 декабря — разбейте на две строки",IF($B5&lt;$A5,"Конец периода раньше начала",IF($E5="","Ставка на эту дату не найдена: дополните таблицу ставок",""))))</f>
+        <f>IF($A5="","",IF(YEAR($A5)&lt;&gt;YEAR($B5),"Период пересекает 31 декабря — разбейте на две строки",IF($B5&lt;$A5,"Конец периода раньше начала",IF(OR($B4="",$A5&lt;&gt;$B4+1),"Период пропущен или перекрыт — исправьте даты",IF($E5="","Ставка на эту дату не найдена: дополните таблицу ставок","")))))</f>
         <v/>
       </c>
     </row>
@@ -917,7 +924,7 @@
         <v/>
       </c>
       <c r="D6" s="11">
-        <f>IF($A6="","",'Входные данные'!$B$4-SUMIF('Входные данные'!$A$35:$A$44,"&lt;="&amp;$A6,'Входные данные'!$B$35:$B$44))</f>
+        <f>IF($A6="","",'Входные данные'!$B$4-SUMIF('Входные данные'!$A$35:$A$44,"&lt;"&amp;$A6,'Входные данные'!$B$35:$B$44))</f>
         <v/>
       </c>
       <c r="E6" s="12">
@@ -933,7 +940,7 @@
         <v/>
       </c>
       <c r="H6" s="13">
-        <f>IF($A6="","",IF(YEAR($A6)&lt;&gt;YEAR($B6),"Период пересекает 31 декабря — разбейте на две строки",IF($B6&lt;$A6,"Конец периода раньше начала",IF($E6="","Ставка на эту дату не найдена: дополните таблицу ставок",""))))</f>
+        <f>IF($A6="","",IF(YEAR($A6)&lt;&gt;YEAR($B6),"Период пересекает 31 декабря — разбейте на две строки",IF($B6&lt;$A6,"Конец периода раньше начала",IF(OR($B5="",$A6&lt;&gt;$B5+1),"Период пропущен или перекрыт — исправьте даты",IF($E6="","Ставка на эту дату не найдена: дополните таблицу ставок","")))))</f>
         <v/>
       </c>
     </row>
@@ -945,7 +952,7 @@
         <v/>
       </c>
       <c r="D7" s="11">
-        <f>IF($A7="","",'Входные данные'!$B$4-SUMIF('Входные данные'!$A$35:$A$44,"&lt;="&amp;$A7,'Входные данные'!$B$35:$B$44))</f>
+        <f>IF($A7="","",'Входные данные'!$B$4-SUMIF('Входные данные'!$A$35:$A$44,"&lt;"&amp;$A7,'Входные данные'!$B$35:$B$44))</f>
         <v/>
       </c>
       <c r="E7" s="12">
@@ -961,7 +968,7 @@
         <v/>
       </c>
       <c r="H7" s="13">
-        <f>IF($A7="","",IF(YEAR($A7)&lt;&gt;YEAR($B7),"Период пересекает 31 декабря — разбейте на две строки",IF($B7&lt;$A7,"Конец периода раньше начала",IF($E7="","Ставка на эту дату не найдена: дополните таблицу ставок",""))))</f>
+        <f>IF($A7="","",IF(YEAR($A7)&lt;&gt;YEAR($B7),"Период пересекает 31 декабря — разбейте на две строки",IF($B7&lt;$A7,"Конец периода раньше начала",IF(OR($B6="",$A7&lt;&gt;$B6+1),"Период пропущен или перекрыт — исправьте даты",IF($E7="","Ставка на эту дату не найдена: дополните таблицу ставок","")))))</f>
         <v/>
       </c>
     </row>
@@ -973,7 +980,7 @@
         <v/>
       </c>
       <c r="D8" s="11">
-        <f>IF($A8="","",'Входные данные'!$B$4-SUMIF('Входные данные'!$A$35:$A$44,"&lt;="&amp;$A8,'Входные данные'!$B$35:$B$44))</f>
+        <f>IF($A8="","",'Входные данные'!$B$4-SUMIF('Входные данные'!$A$35:$A$44,"&lt;"&amp;$A8,'Входные данные'!$B$35:$B$44))</f>
         <v/>
       </c>
       <c r="E8" s="12">
@@ -989,7 +996,7 @@
         <v/>
       </c>
       <c r="H8" s="13">
-        <f>IF($A8="","",IF(YEAR($A8)&lt;&gt;YEAR($B8),"Период пересекает 31 декабря — разбейте на две строки",IF($B8&lt;$A8,"Конец периода раньше начала",IF($E8="","Ставка на эту дату не найдена: дополните таблицу ставок",""))))</f>
+        <f>IF($A8="","",IF(YEAR($A8)&lt;&gt;YEAR($B8),"Период пересекает 31 декабря — разбейте на две строки",IF($B8&lt;$A8,"Конец периода раньше начала",IF(OR($B7="",$A8&lt;&gt;$B7+1),"Период пропущен или перекрыт — исправьте даты",IF($E8="","Ставка на эту дату не найдена: дополните таблицу ставок","")))))</f>
         <v/>
       </c>
     </row>
@@ -1001,7 +1008,7 @@
         <v/>
       </c>
       <c r="D9" s="11">
-        <f>IF($A9="","",'Входные данные'!$B$4-SUMIF('Входные данные'!$A$35:$A$44,"&lt;="&amp;$A9,'Входные данные'!$B$35:$B$44))</f>
+        <f>IF($A9="","",'Входные данные'!$B$4-SUMIF('Входные данные'!$A$35:$A$44,"&lt;"&amp;$A9,'Входные данные'!$B$35:$B$44))</f>
         <v/>
       </c>
       <c r="E9" s="12">
@@ -1017,7 +1024,7 @@
         <v/>
       </c>
       <c r="H9" s="13">
-        <f>IF($A9="","",IF(YEAR($A9)&lt;&gt;YEAR($B9),"Период пересекает 31 декабря — разбейте на две строки",IF($B9&lt;$A9,"Конец периода раньше начала",IF($E9="","Ставка на эту дату не найдена: дополните таблицу ставок",""))))</f>
+        <f>IF($A9="","",IF(YEAR($A9)&lt;&gt;YEAR($B9),"Период пересекает 31 декабря — разбейте на две строки",IF($B9&lt;$A9,"Конец периода раньше начала",IF(OR($B8="",$A9&lt;&gt;$B8+1),"Период пропущен или перекрыт — исправьте даты",IF($E9="","Ставка на эту дату не найдена: дополните таблицу ставок","")))))</f>
         <v/>
       </c>
     </row>
@@ -1029,7 +1036,7 @@
         <v/>
       </c>
       <c r="D10" s="11">
-        <f>IF($A10="","",'Входные данные'!$B$4-SUMIF('Входные данные'!$A$35:$A$44,"&lt;="&amp;$A10,'Входные данные'!$B$35:$B$44))</f>
+        <f>IF($A10="","",'Входные данные'!$B$4-SUMIF('Входные данные'!$A$35:$A$44,"&lt;"&amp;$A10,'Входные данные'!$B$35:$B$44))</f>
         <v/>
       </c>
       <c r="E10" s="12">
@@ -1045,7 +1052,7 @@
         <v/>
       </c>
       <c r="H10" s="13">
-        <f>IF($A10="","",IF(YEAR($A10)&lt;&gt;YEAR($B10),"Период пересекает 31 декабря — разбейте на две строки",IF($B10&lt;$A10,"Конец периода раньше начала",IF($E10="","Ставка на эту дату не найдена: дополните таблицу ставок",""))))</f>
+        <f>IF($A10="","",IF(YEAR($A10)&lt;&gt;YEAR($B10),"Период пересекает 31 декабря — разбейте на две строки",IF($B10&lt;$A10,"Конец периода раньше начала",IF(OR($B9="",$A10&lt;&gt;$B9+1),"Период пропущен или перекрыт — исправьте даты",IF($E10="","Ставка на эту дату не найдена: дополните таблицу ставок","")))))</f>
         <v/>
       </c>
     </row>
@@ -1057,7 +1064,7 @@
         <v/>
       </c>
       <c r="D11" s="11">
-        <f>IF($A11="","",'Входные данные'!$B$4-SUMIF('Входные данные'!$A$35:$A$44,"&lt;="&amp;$A11,'Входные данные'!$B$35:$B$44))</f>
+        <f>IF($A11="","",'Входные данные'!$B$4-SUMIF('Входные данные'!$A$35:$A$44,"&lt;"&amp;$A11,'Входные данные'!$B$35:$B$44))</f>
         <v/>
       </c>
       <c r="E11" s="12">
@@ -1073,7 +1080,7 @@
         <v/>
       </c>
       <c r="H11" s="13">
-        <f>IF($A11="","",IF(YEAR($A11)&lt;&gt;YEAR($B11),"Период пересекает 31 декабря — разбейте на две строки",IF($B11&lt;$A11,"Конец периода раньше начала",IF($E11="","Ставка на эту дату не найдена: дополните таблицу ставок",""))))</f>
+        <f>IF($A11="","",IF(YEAR($A11)&lt;&gt;YEAR($B11),"Период пересекает 31 декабря — разбейте на две строки",IF($B11&lt;$A11,"Конец периода раньше начала",IF(OR($B10="",$A11&lt;&gt;$B10+1),"Период пропущен или перекрыт — исправьте даты",IF($E11="","Ставка на эту дату не найдена: дополните таблицу ставок","")))))</f>
         <v/>
       </c>
     </row>
@@ -1085,7 +1092,7 @@
         <v/>
       </c>
       <c r="D12" s="11">
-        <f>IF($A12="","",'Входные данные'!$B$4-SUMIF('Входные данные'!$A$35:$A$44,"&lt;="&amp;$A12,'Входные данные'!$B$35:$B$44))</f>
+        <f>IF($A12="","",'Входные данные'!$B$4-SUMIF('Входные данные'!$A$35:$A$44,"&lt;"&amp;$A12,'Входные данные'!$B$35:$B$44))</f>
         <v/>
       </c>
       <c r="E12" s="12">
@@ -1101,7 +1108,7 @@
         <v/>
       </c>
       <c r="H12" s="13">
-        <f>IF($A12="","",IF(YEAR($A12)&lt;&gt;YEAR($B12),"Период пересекает 31 декабря — разбейте на две строки",IF($B12&lt;$A12,"Конец периода раньше начала",IF($E12="","Ставка на эту дату не найдена: дополните таблицу ставок",""))))</f>
+        <f>IF($A12="","",IF(YEAR($A12)&lt;&gt;YEAR($B12),"Период пересекает 31 декабря — разбейте на две строки",IF($B12&lt;$A12,"Конец периода раньше начала",IF(OR($B11="",$A12&lt;&gt;$B11+1),"Период пропущен или перекрыт — исправьте даты",IF($E12="","Ставка на эту дату не найдена: дополните таблицу ставок","")))))</f>
         <v/>
       </c>
     </row>
@@ -1113,7 +1120,7 @@
         <v/>
       </c>
       <c r="D13" s="11">
-        <f>IF($A13="","",'Входные данные'!$B$4-SUMIF('Входные данные'!$A$35:$A$44,"&lt;="&amp;$A13,'Входные данные'!$B$35:$B$44))</f>
+        <f>IF($A13="","",'Входные данные'!$B$4-SUMIF('Входные данные'!$A$35:$A$44,"&lt;"&amp;$A13,'Входные данные'!$B$35:$B$44))</f>
         <v/>
       </c>
       <c r="E13" s="12">
@@ -1129,7 +1136,7 @@
         <v/>
       </c>
       <c r="H13" s="13">
-        <f>IF($A13="","",IF(YEAR($A13)&lt;&gt;YEAR($B13),"Период пересекает 31 декабря — разбейте на две строки",IF($B13&lt;$A13,"Конец периода раньше начала",IF($E13="","Ставка на эту дату не найдена: дополните таблицу ставок",""))))</f>
+        <f>IF($A13="","",IF(YEAR($A13)&lt;&gt;YEAR($B13),"Период пересекает 31 декабря — разбейте на две строки",IF($B13&lt;$A13,"Конец периода раньше начала",IF(OR($B12="",$A13&lt;&gt;$B12+1),"Период пропущен или перекрыт — исправьте даты",IF($E13="","Ставка на эту дату не найдена: дополните таблицу ставок","")))))</f>
         <v/>
       </c>
     </row>
@@ -1141,7 +1148,7 @@
         <v/>
       </c>
       <c r="D14" s="11">
-        <f>IF($A14="","",'Входные данные'!$B$4-SUMIF('Входные данные'!$A$35:$A$44,"&lt;="&amp;$A14,'Входные данные'!$B$35:$B$44))</f>
+        <f>IF($A14="","",'Входные данные'!$B$4-SUMIF('Входные данные'!$A$35:$A$44,"&lt;"&amp;$A14,'Входные данные'!$B$35:$B$44))</f>
         <v/>
       </c>
       <c r="E14" s="12">
@@ -1157,7 +1164,7 @@
         <v/>
       </c>
       <c r="H14" s="13">
-        <f>IF($A14="","",IF(YEAR($A14)&lt;&gt;YEAR($B14),"Период пересекает 31 декабря — разбейте на две строки",IF($B14&lt;$A14,"Конец периода раньше начала",IF($E14="","Ставка на эту дату не найдена: дополните таблицу ставок",""))))</f>
+        <f>IF($A14="","",IF(YEAR($A14)&lt;&gt;YEAR($B14),"Период пересекает 31 декабря — разбейте на две строки",IF($B14&lt;$A14,"Конец периода раньше начала",IF(OR($B13="",$A14&lt;&gt;$B13+1),"Период пропущен или перекрыт — исправьте даты",IF($E14="","Ставка на эту дату не найдена: дополните таблицу ставок","")))))</f>
         <v/>
       </c>
     </row>
@@ -1169,7 +1176,7 @@
         <v/>
       </c>
       <c r="D15" s="11">
-        <f>IF($A15="","",'Входные данные'!$B$4-SUMIF('Входные данные'!$A$35:$A$44,"&lt;="&amp;$A15,'Входные данные'!$B$35:$B$44))</f>
+        <f>IF($A15="","",'Входные данные'!$B$4-SUMIF('Входные данные'!$A$35:$A$44,"&lt;"&amp;$A15,'Входные данные'!$B$35:$B$44))</f>
         <v/>
       </c>
       <c r="E15" s="12">
@@ -1185,7 +1192,7 @@
         <v/>
       </c>
       <c r="H15" s="13">
-        <f>IF($A15="","",IF(YEAR($A15)&lt;&gt;YEAR($B15),"Период пересекает 31 декабря — разбейте на две строки",IF($B15&lt;$A15,"Конец периода раньше начала",IF($E15="","Ставка на эту дату не найдена: дополните таблицу ставок",""))))</f>
+        <f>IF($A15="","",IF(YEAR($A15)&lt;&gt;YEAR($B15),"Период пересекает 31 декабря — разбейте на две строки",IF($B15&lt;$A15,"Конец периода раньше начала",IF(OR($B14="",$A15&lt;&gt;$B14+1),"Период пропущен или перекрыт — исправьте даты",IF($E15="","Ставка на эту дату не найдена: дополните таблицу ставок","")))))</f>
         <v/>
       </c>
     </row>
@@ -1197,7 +1204,7 @@
         <v/>
       </c>
       <c r="D16" s="11">
-        <f>IF($A16="","",'Входные данные'!$B$4-SUMIF('Входные данные'!$A$35:$A$44,"&lt;="&amp;$A16,'Входные данные'!$B$35:$B$44))</f>
+        <f>IF($A16="","",'Входные данные'!$B$4-SUMIF('Входные данные'!$A$35:$A$44,"&lt;"&amp;$A16,'Входные данные'!$B$35:$B$44))</f>
         <v/>
       </c>
       <c r="E16" s="12">
@@ -1213,7 +1220,7 @@
         <v/>
       </c>
       <c r="H16" s="13">
-        <f>IF($A16="","",IF(YEAR($A16)&lt;&gt;YEAR($B16),"Период пересекает 31 декабря — разбейте на две строки",IF($B16&lt;$A16,"Конец периода раньше начала",IF($E16="","Ставка на эту дату не найдена: дополните таблицу ставок",""))))</f>
+        <f>IF($A16="","",IF(YEAR($A16)&lt;&gt;YEAR($B16),"Период пересекает 31 декабря — разбейте на две строки",IF($B16&lt;$A16,"Конец периода раньше начала",IF(OR($B15="",$A16&lt;&gt;$B15+1),"Период пропущен или перекрыт — исправьте даты",IF($E16="","Ставка на эту дату не найдена: дополните таблицу ставок","")))))</f>
         <v/>
       </c>
     </row>
@@ -1225,7 +1232,7 @@
         <v/>
       </c>
       <c r="D17" s="11">
-        <f>IF($A17="","",'Входные данные'!$B$4-SUMIF('Входные данные'!$A$35:$A$44,"&lt;="&amp;$A17,'Входные данные'!$B$35:$B$44))</f>
+        <f>IF($A17="","",'Входные данные'!$B$4-SUMIF('Входные данные'!$A$35:$A$44,"&lt;"&amp;$A17,'Входные данные'!$B$35:$B$44))</f>
         <v/>
       </c>
       <c r="E17" s="12">
@@ -1241,7 +1248,7 @@
         <v/>
       </c>
       <c r="H17" s="13">
-        <f>IF($A17="","",IF(YEAR($A17)&lt;&gt;YEAR($B17),"Период пересекает 31 декабря — разбейте на две строки",IF($B17&lt;$A17,"Конец периода раньше начала",IF($E17="","Ставка на эту дату не найдена: дополните таблицу ставок",""))))</f>
+        <f>IF($A17="","",IF(YEAR($A17)&lt;&gt;YEAR($B17),"Период пересекает 31 декабря — разбейте на две строки",IF($B17&lt;$A17,"Конец периода раньше начала",IF(OR($B16="",$A17&lt;&gt;$B16+1),"Период пропущен или перекрыт — исправьте даты",IF($E17="","Ставка на эту дату не найдена: дополните таблицу ставок","")))))</f>
         <v/>
       </c>
     </row>
@@ -1253,7 +1260,7 @@
         <v/>
       </c>
       <c r="D18" s="11">
-        <f>IF($A18="","",'Входные данные'!$B$4-SUMIF('Входные данные'!$A$35:$A$44,"&lt;="&amp;$A18,'Входные данные'!$B$35:$B$44))</f>
+        <f>IF($A18="","",'Входные данные'!$B$4-SUMIF('Входные данные'!$A$35:$A$44,"&lt;"&amp;$A18,'Входные данные'!$B$35:$B$44))</f>
         <v/>
       </c>
       <c r="E18" s="12">
@@ -1269,7 +1276,7 @@
         <v/>
       </c>
       <c r="H18" s="13">
-        <f>IF($A18="","",IF(YEAR($A18)&lt;&gt;YEAR($B18),"Период пересекает 31 декабря — разбейте на две строки",IF($B18&lt;$A18,"Конец периода раньше начала",IF($E18="","Ставка на эту дату не найдена: дополните таблицу ставок",""))))</f>
+        <f>IF($A18="","",IF(YEAR($A18)&lt;&gt;YEAR($B18),"Период пересекает 31 декабря — разбейте на две строки",IF($B18&lt;$A18,"Конец периода раньше начала",IF(OR($B17="",$A18&lt;&gt;$B17+1),"Период пропущен или перекрыт — исправьте даты",IF($E18="","Ставка на эту дату не найдена: дополните таблицу ставок","")))))</f>
         <v/>
       </c>
     </row>
@@ -1281,7 +1288,7 @@
         <v/>
       </c>
       <c r="D19" s="11">
-        <f>IF($A19="","",'Входные данные'!$B$4-SUMIF('Входные данные'!$A$35:$A$44,"&lt;="&amp;$A19,'Входные данные'!$B$35:$B$44))</f>
+        <f>IF($A19="","",'Входные данные'!$B$4-SUMIF('Входные данные'!$A$35:$A$44,"&lt;"&amp;$A19,'Входные данные'!$B$35:$B$44))</f>
         <v/>
       </c>
       <c r="E19" s="12">
@@ -1297,7 +1304,7 @@
         <v/>
       </c>
       <c r="H19" s="13">
-        <f>IF($A19="","",IF(YEAR($A19)&lt;&gt;YEAR($B19),"Период пересекает 31 декабря — разбейте на две строки",IF($B19&lt;$A19,"Конец периода раньше начала",IF($E19="","Ставка на эту дату не найдена: дополните таблицу ставок",""))))</f>
+        <f>IF($A19="","",IF(YEAR($A19)&lt;&gt;YEAR($B19),"Период пересекает 31 декабря — разбейте на две строки",IF($B19&lt;$A19,"Конец периода раньше начала",IF(OR($B18="",$A19&lt;&gt;$B18+1),"Период пропущен или перекрыт — исправьте даты",IF($E19="","Ставка на эту дату не найдена: дополните таблицу ставок","")))))</f>
         <v/>
       </c>
     </row>
@@ -1309,7 +1316,7 @@
         <v/>
       </c>
       <c r="D20" s="11">
-        <f>IF($A20="","",'Входные данные'!$B$4-SUMIF('Входные данные'!$A$35:$A$44,"&lt;="&amp;$A20,'Входные данные'!$B$35:$B$44))</f>
+        <f>IF($A20="","",'Входные данные'!$B$4-SUMIF('Входные данные'!$A$35:$A$44,"&lt;"&amp;$A20,'Входные данные'!$B$35:$B$44))</f>
         <v/>
       </c>
       <c r="E20" s="12">
@@ -1325,7 +1332,7 @@
         <v/>
       </c>
       <c r="H20" s="13">
-        <f>IF($A20="","",IF(YEAR($A20)&lt;&gt;YEAR($B20),"Период пересекает 31 декабря — разбейте на две строки",IF($B20&lt;$A20,"Конец периода раньше начала",IF($E20="","Ставка на эту дату не найдена: дополните таблицу ставок",""))))</f>
+        <f>IF($A20="","",IF(YEAR($A20)&lt;&gt;YEAR($B20),"Период пересекает 31 декабря — разбейте на две строки",IF($B20&lt;$A20,"Конец периода раньше начала",IF(OR($B19="",$A20&lt;&gt;$B19+1),"Период пропущен или перекрыт — исправьте даты",IF($E20="","Ставка на эту дату не найдена: дополните таблицу ставок","")))))</f>
         <v/>
       </c>
     </row>
@@ -1337,7 +1344,7 @@
         <v/>
       </c>
       <c r="D21" s="11">
-        <f>IF($A21="","",'Входные данные'!$B$4-SUMIF('Входные данные'!$A$35:$A$44,"&lt;="&amp;$A21,'Входные данные'!$B$35:$B$44))</f>
+        <f>IF($A21="","",'Входные данные'!$B$4-SUMIF('Входные данные'!$A$35:$A$44,"&lt;"&amp;$A21,'Входные данные'!$B$35:$B$44))</f>
         <v/>
       </c>
       <c r="E21" s="12">
@@ -1353,7 +1360,7 @@
         <v/>
       </c>
       <c r="H21" s="13">
-        <f>IF($A21="","",IF(YEAR($A21)&lt;&gt;YEAR($B21),"Период пересекает 31 декабря — разбейте на две строки",IF($B21&lt;$A21,"Конец периода раньше начала",IF($E21="","Ставка на эту дату не найдена: дополните таблицу ставок",""))))</f>
+        <f>IF($A21="","",IF(YEAR($A21)&lt;&gt;YEAR($B21),"Период пересекает 31 декабря — разбейте на две строки",IF($B21&lt;$A21,"Конец периода раньше начала",IF(OR($B20="",$A21&lt;&gt;$B20+1),"Период пропущен или перекрыт — исправьте даты",IF($E21="","Ставка на эту дату не найдена: дополните таблицу ставок","")))))</f>
         <v/>
       </c>
     </row>
@@ -1365,7 +1372,7 @@
         <v/>
       </c>
       <c r="D22" s="11">
-        <f>IF($A22="","",'Входные данные'!$B$4-SUMIF('Входные данные'!$A$35:$A$44,"&lt;="&amp;$A22,'Входные данные'!$B$35:$B$44))</f>
+        <f>IF($A22="","",'Входные данные'!$B$4-SUMIF('Входные данные'!$A$35:$A$44,"&lt;"&amp;$A22,'Входные данные'!$B$35:$B$44))</f>
         <v/>
       </c>
       <c r="E22" s="12">
@@ -1381,7 +1388,7 @@
         <v/>
       </c>
       <c r="H22" s="13">
-        <f>IF($A22="","",IF(YEAR($A22)&lt;&gt;YEAR($B22),"Период пересекает 31 декабря — разбейте на две строки",IF($B22&lt;$A22,"Конец периода раньше начала",IF($E22="","Ставка на эту дату не найдена: дополните таблицу ставок",""))))</f>
+        <f>IF($A22="","",IF(YEAR($A22)&lt;&gt;YEAR($B22),"Период пересекает 31 декабря — разбейте на две строки",IF($B22&lt;$A22,"Конец периода раньше начала",IF(OR($B21="",$A22&lt;&gt;$B21+1),"Период пропущен или перекрыт — исправьте даты",IF($E22="","Ставка на эту дату не найдена: дополните таблицу ставок","")))))</f>
         <v/>
       </c>
     </row>
@@ -1393,7 +1400,7 @@
         <v/>
       </c>
       <c r="D23" s="11">
-        <f>IF($A23="","",'Входные данные'!$B$4-SUMIF('Входные данные'!$A$35:$A$44,"&lt;="&amp;$A23,'Входные данные'!$B$35:$B$44))</f>
+        <f>IF($A23="","",'Входные данные'!$B$4-SUMIF('Входные данные'!$A$35:$A$44,"&lt;"&amp;$A23,'Входные данные'!$B$35:$B$44))</f>
         <v/>
       </c>
       <c r="E23" s="12">
@@ -1409,7 +1416,7 @@
         <v/>
       </c>
       <c r="H23" s="13">
-        <f>IF($A23="","",IF(YEAR($A23)&lt;&gt;YEAR($B23),"Период пересекает 31 декабря — разбейте на две строки",IF($B23&lt;$A23,"Конец периода раньше начала",IF($E23="","Ставка на эту дату не найдена: дополните таблицу ставок",""))))</f>
+        <f>IF($A23="","",IF(YEAR($A23)&lt;&gt;YEAR($B23),"Период пересекает 31 декабря — разбейте на две строки",IF($B23&lt;$A23,"Конец периода раньше начала",IF(OR($B22="",$A23&lt;&gt;$B22+1),"Период пропущен или перекрыт — исправьте даты",IF($E23="","Ставка на эту дату не найдена: дополните таблицу ставок","")))))</f>
         <v/>
       </c>
     </row>
@@ -1421,7 +1428,7 @@
         <v/>
       </c>
       <c r="D24" s="11">
-        <f>IF($A24="","",'Входные данные'!$B$4-SUMIF('Входные данные'!$A$35:$A$44,"&lt;="&amp;$A24,'Входные данные'!$B$35:$B$44))</f>
+        <f>IF($A24="","",'Входные данные'!$B$4-SUMIF('Входные данные'!$A$35:$A$44,"&lt;"&amp;$A24,'Входные данные'!$B$35:$B$44))</f>
         <v/>
       </c>
       <c r="E24" s="12">
@@ -1437,7 +1444,7 @@
         <v/>
       </c>
       <c r="H24" s="13">
-        <f>IF($A24="","",IF(YEAR($A24)&lt;&gt;YEAR($B24),"Период пересекает 31 декабря — разбейте на две строки",IF($B24&lt;$A24,"Конец периода раньше начала",IF($E24="","Ставка на эту дату не найдена: дополните таблицу ставок",""))))</f>
+        <f>IF($A24="","",IF(YEAR($A24)&lt;&gt;YEAR($B24),"Период пересекает 31 декабря — разбейте на две строки",IF($B24&lt;$A24,"Конец периода раньше начала",IF(OR($B23="",$A24&lt;&gt;$B23+1),"Период пропущен или перекрыт — исправьте даты",IF($E24="","Ставка на эту дату не найдена: дополните таблицу ставок","")))))</f>
         <v/>
       </c>
     </row>
@@ -1449,7 +1456,7 @@
         <v/>
       </c>
       <c r="D25" s="11">
-        <f>IF($A25="","",'Входные данные'!$B$4-SUMIF('Входные данные'!$A$35:$A$44,"&lt;="&amp;$A25,'Входные данные'!$B$35:$B$44))</f>
+        <f>IF($A25="","",'Входные данные'!$B$4-SUMIF('Входные данные'!$A$35:$A$44,"&lt;"&amp;$A25,'Входные данные'!$B$35:$B$44))</f>
         <v/>
       </c>
       <c r="E25" s="12">
@@ -1465,7 +1472,7 @@
         <v/>
       </c>
       <c r="H25" s="13">
-        <f>IF($A25="","",IF(YEAR($A25)&lt;&gt;YEAR($B25),"Период пересекает 31 декабря — разбейте на две строки",IF($B25&lt;$A25,"Конец периода раньше начала",IF($E25="","Ставка на эту дату не найдена: дополните таблицу ставок",""))))</f>
+        <f>IF($A25="","",IF(YEAR($A25)&lt;&gt;YEAR($B25),"Период пересекает 31 декабря — разбейте на две строки",IF($B25&lt;$A25,"Конец периода раньше начала",IF(OR($B24="",$A25&lt;&gt;$B24+1),"Период пропущен или перекрыт — исправьте даты",IF($E25="","Ставка на эту дату не найдена: дополните таблицу ставок","")))))</f>
         <v/>
       </c>
     </row>
@@ -1477,7 +1484,7 @@
         <v/>
       </c>
       <c r="D26" s="11">
-        <f>IF($A26="","",'Входные данные'!$B$4-SUMIF('Входные данные'!$A$35:$A$44,"&lt;="&amp;$A26,'Входные данные'!$B$35:$B$44))</f>
+        <f>IF($A26="","",'Входные данные'!$B$4-SUMIF('Входные данные'!$A$35:$A$44,"&lt;"&amp;$A26,'Входные данные'!$B$35:$B$44))</f>
         <v/>
       </c>
       <c r="E26" s="12">
@@ -1493,7 +1500,7 @@
         <v/>
       </c>
       <c r="H26" s="13">
-        <f>IF($A26="","",IF(YEAR($A26)&lt;&gt;YEAR($B26),"Период пересекает 31 декабря — разбейте на две строки",IF($B26&lt;$A26,"Конец периода раньше начала",IF($E26="","Ставка на эту дату не найдена: дополните таблицу ставок",""))))</f>
+        <f>IF($A26="","",IF(YEAR($A26)&lt;&gt;YEAR($B26),"Период пересекает 31 декабря — разбейте на две строки",IF($B26&lt;$A26,"Конец периода раньше начала",IF(OR($B25="",$A26&lt;&gt;$B25+1),"Период пропущен или перекрыт — исправьте даты",IF($E26="","Ставка на эту дату не найдена: дополните таблицу ставок","")))))</f>
         <v/>
       </c>
     </row>
@@ -1505,7 +1512,7 @@
         <v/>
       </c>
       <c r="D27" s="11">
-        <f>IF($A27="","",'Входные данные'!$B$4-SUMIF('Входные данные'!$A$35:$A$44,"&lt;="&amp;$A27,'Входные данные'!$B$35:$B$44))</f>
+        <f>IF($A27="","",'Входные данные'!$B$4-SUMIF('Входные данные'!$A$35:$A$44,"&lt;"&amp;$A27,'Входные данные'!$B$35:$B$44))</f>
         <v/>
       </c>
       <c r="E27" s="12">
@@ -1521,7 +1528,7 @@
         <v/>
       </c>
       <c r="H27" s="13">
-        <f>IF($A27="","",IF(YEAR($A27)&lt;&gt;YEAR($B27),"Период пересекает 31 декабря — разбейте на две строки",IF($B27&lt;$A27,"Конец периода раньше начала",IF($E27="","Ставка на эту дату не найдена: дополните таблицу ставок",""))))</f>
+        <f>IF($A27="","",IF(YEAR($A27)&lt;&gt;YEAR($B27),"Период пересекает 31 декабря — разбейте на две строки",IF($B27&lt;$A27,"Конец периода раньше начала",IF(OR($B26="",$A27&lt;&gt;$B26+1),"Период пропущен или перекрыт — исправьте даты",IF($E27="","Ставка на эту дату не найдена: дополните таблицу ставок","")))))</f>
         <v/>
       </c>
     </row>
@@ -1533,7 +1540,7 @@
         <v/>
       </c>
       <c r="D28" s="11">
-        <f>IF($A28="","",'Входные данные'!$B$4-SUMIF('Входные данные'!$A$35:$A$44,"&lt;="&amp;$A28,'Входные данные'!$B$35:$B$44))</f>
+        <f>IF($A28="","",'Входные данные'!$B$4-SUMIF('Входные данные'!$A$35:$A$44,"&lt;"&amp;$A28,'Входные данные'!$B$35:$B$44))</f>
         <v/>
       </c>
       <c r="E28" s="12">
@@ -1549,7 +1556,7 @@
         <v/>
       </c>
       <c r="H28" s="13">
-        <f>IF($A28="","",IF(YEAR($A28)&lt;&gt;YEAR($B28),"Период пересекает 31 декабря — разбейте на две строки",IF($B28&lt;$A28,"Конец периода раньше начала",IF($E28="","Ставка на эту дату не найдена: дополните таблицу ставок",""))))</f>
+        <f>IF($A28="","",IF(YEAR($A28)&lt;&gt;YEAR($B28),"Период пересекает 31 декабря — разбейте на две строки",IF($B28&lt;$A28,"Конец периода раньше начала",IF(OR($B27="",$A28&lt;&gt;$B27+1),"Период пропущен или перекрыт — исправьте даты",IF($E28="","Ставка на эту дату не найдена: дополните таблицу ставок","")))))</f>
         <v/>
       </c>
     </row>
@@ -1561,7 +1568,7 @@
         <v/>
       </c>
       <c r="D29" s="11">
-        <f>IF($A29="","",'Входные данные'!$B$4-SUMIF('Входные данные'!$A$35:$A$44,"&lt;="&amp;$A29,'Входные данные'!$B$35:$B$44))</f>
+        <f>IF($A29="","",'Входные данные'!$B$4-SUMIF('Входные данные'!$A$35:$A$44,"&lt;"&amp;$A29,'Входные данные'!$B$35:$B$44))</f>
         <v/>
       </c>
       <c r="E29" s="12">
@@ -1577,7 +1584,7 @@
         <v/>
       </c>
       <c r="H29" s="13">
-        <f>IF($A29="","",IF(YEAR($A29)&lt;&gt;YEAR($B29),"Период пересекает 31 декабря — разбейте на две строки",IF($B29&lt;$A29,"Конец периода раньше начала",IF($E29="","Ставка на эту дату не найдена: дополните таблицу ставок",""))))</f>
+        <f>IF($A29="","",IF(YEAR($A29)&lt;&gt;YEAR($B29),"Период пересекает 31 декабря — разбейте на две строки",IF($B29&lt;$A29,"Конец периода раньше начала",IF(OR($B28="",$A29&lt;&gt;$B28+1),"Период пропущен или перекрыт — исправьте даты",IF($E29="","Ставка на эту дату не найдена: дополните таблицу ставок","")))))</f>
         <v/>
       </c>
     </row>
@@ -1589,7 +1596,7 @@
         <v/>
       </c>
       <c r="D30" s="11">
-        <f>IF($A30="","",'Входные данные'!$B$4-SUMIF('Входные данные'!$A$35:$A$44,"&lt;="&amp;$A30,'Входные данные'!$B$35:$B$44))</f>
+        <f>IF($A30="","",'Входные данные'!$B$4-SUMIF('Входные данные'!$A$35:$A$44,"&lt;"&amp;$A30,'Входные данные'!$B$35:$B$44))</f>
         <v/>
       </c>
       <c r="E30" s="12">
@@ -1605,7 +1612,7 @@
         <v/>
       </c>
       <c r="H30" s="13">
-        <f>IF($A30="","",IF(YEAR($A30)&lt;&gt;YEAR($B30),"Период пересекает 31 декабря — разбейте на две строки",IF($B30&lt;$A30,"Конец периода раньше начала",IF($E30="","Ставка на эту дату не найдена: дополните таблицу ставок",""))))</f>
+        <f>IF($A30="","",IF(YEAR($A30)&lt;&gt;YEAR($B30),"Период пересекает 31 декабря — разбейте на две строки",IF($B30&lt;$A30,"Конец периода раньше начала",IF(OR($B29="",$A30&lt;&gt;$B29+1),"Период пропущен или перекрыт — исправьте даты",IF($E30="","Ставка на эту дату не найдена: дополните таблицу ставок","")))))</f>
         <v/>
       </c>
     </row>
@@ -1617,7 +1624,7 @@
         <v/>
       </c>
       <c r="D31" s="11">
-        <f>IF($A31="","",'Входные данные'!$B$4-SUMIF('Входные данные'!$A$35:$A$44,"&lt;="&amp;$A31,'Входные данные'!$B$35:$B$44))</f>
+        <f>IF($A31="","",'Входные данные'!$B$4-SUMIF('Входные данные'!$A$35:$A$44,"&lt;"&amp;$A31,'Входные данные'!$B$35:$B$44))</f>
         <v/>
       </c>
       <c r="E31" s="12">
@@ -1633,7 +1640,7 @@
         <v/>
       </c>
       <c r="H31" s="13">
-        <f>IF($A31="","",IF(YEAR($A31)&lt;&gt;YEAR($B31),"Период пересекает 31 декабря — разбейте на две строки",IF($B31&lt;$A31,"Конец периода раньше начала",IF($E31="","Ставка на эту дату не найдена: дополните таблицу ставок",""))))</f>
+        <f>IF($A31="","",IF(YEAR($A31)&lt;&gt;YEAR($B31),"Период пересекает 31 декабря — разбейте на две строки",IF($B31&lt;$A31,"Конец периода раньше начала",IF(OR($B30="",$A31&lt;&gt;$B30+1),"Период пропущен или перекрыт — исправьте даты",IF($E31="","Ставка на эту дату не найдена: дополните таблицу ставок","")))))</f>
         <v/>
       </c>
     </row>
@@ -1645,7 +1652,7 @@
         <v/>
       </c>
       <c r="D32" s="11">
-        <f>IF($A32="","",'Входные данные'!$B$4-SUMIF('Входные данные'!$A$35:$A$44,"&lt;="&amp;$A32,'Входные данные'!$B$35:$B$44))</f>
+        <f>IF($A32="","",'Входные данные'!$B$4-SUMIF('Входные данные'!$A$35:$A$44,"&lt;"&amp;$A32,'Входные данные'!$B$35:$B$44))</f>
         <v/>
       </c>
       <c r="E32" s="12">
@@ -1661,7 +1668,7 @@
         <v/>
       </c>
       <c r="H32" s="13">
-        <f>IF($A32="","",IF(YEAR($A32)&lt;&gt;YEAR($B32),"Период пересекает 31 декабря — разбейте на две строки",IF($B32&lt;$A32,"Конец периода раньше начала",IF($E32="","Ставка на эту дату не найдена: дополните таблицу ставок",""))))</f>
+        <f>IF($A32="","",IF(YEAR($A32)&lt;&gt;YEAR($B32),"Период пересекает 31 декабря — разбейте на две строки",IF($B32&lt;$A32,"Конец периода раньше начала",IF(OR($B31="",$A32&lt;&gt;$B31+1),"Период пропущен или перекрыт — исправьте даты",IF($E32="","Ставка на эту дату не найдена: дополните таблицу ставок","")))))</f>
         <v/>
       </c>
     </row>
@@ -1673,7 +1680,7 @@
         <v/>
       </c>
       <c r="D33" s="11">
-        <f>IF($A33="","",'Входные данные'!$B$4-SUMIF('Входные данные'!$A$35:$A$44,"&lt;="&amp;$A33,'Входные данные'!$B$35:$B$44))</f>
+        <f>IF($A33="","",'Входные данные'!$B$4-SUMIF('Входные данные'!$A$35:$A$44,"&lt;"&amp;$A33,'Входные данные'!$B$35:$B$44))</f>
         <v/>
       </c>
       <c r="E33" s="12">
@@ -1689,7 +1696,7 @@
         <v/>
       </c>
       <c r="H33" s="13">
-        <f>IF($A33="","",IF(YEAR($A33)&lt;&gt;YEAR($B33),"Период пересекает 31 декабря — разбейте на две строки",IF($B33&lt;$A33,"Конец периода раньше начала",IF($E33="","Ставка на эту дату не найдена: дополните таблицу ставок",""))))</f>
+        <f>IF($A33="","",IF(YEAR($A33)&lt;&gt;YEAR($B33),"Период пересекает 31 декабря — разбейте на две строки",IF($B33&lt;$A33,"Конец периода раньше начала",IF(OR($B32="",$A33&lt;&gt;$B32+1),"Период пропущен или перекрыт — исправьте даты",IF($E33="","Ставка на эту дату не найдена: дополните таблицу ставок","")))))</f>
         <v/>
       </c>
     </row>
@@ -1701,7 +1708,7 @@
         <v/>
       </c>
       <c r="D34" s="11">
-        <f>IF($A34="","",'Входные данные'!$B$4-SUMIF('Входные данные'!$A$35:$A$44,"&lt;="&amp;$A34,'Входные данные'!$B$35:$B$44))</f>
+        <f>IF($A34="","",'Входные данные'!$B$4-SUMIF('Входные данные'!$A$35:$A$44,"&lt;"&amp;$A34,'Входные данные'!$B$35:$B$44))</f>
         <v/>
       </c>
       <c r="E34" s="12">
@@ -1717,7 +1724,7 @@
         <v/>
       </c>
       <c r="H34" s="13">
-        <f>IF($A34="","",IF(YEAR($A34)&lt;&gt;YEAR($B34),"Период пересекает 31 декабря — разбейте на две строки",IF($B34&lt;$A34,"Конец периода раньше начала",IF($E34="","Ставка на эту дату не найдена: дополните таблицу ставок",""))))</f>
+        <f>IF($A34="","",IF(YEAR($A34)&lt;&gt;YEAR($B34),"Период пересекает 31 декабря — разбейте на две строки",IF($B34&lt;$A34,"Конец периода раньше начала",IF(OR($B33="",$A34&lt;&gt;$B33+1),"Период пропущен или перекрыт — исправьте даты",IF($E34="","Ставка на эту дату не найдена: дополните таблицу ставок","")))))</f>
         <v/>
       </c>
     </row>
@@ -1729,7 +1736,7 @@
         <v/>
       </c>
       <c r="D35" s="11">
-        <f>IF($A35="","",'Входные данные'!$B$4-SUMIF('Входные данные'!$A$35:$A$44,"&lt;="&amp;$A35,'Входные данные'!$B$35:$B$44))</f>
+        <f>IF($A35="","",'Входные данные'!$B$4-SUMIF('Входные данные'!$A$35:$A$44,"&lt;"&amp;$A35,'Входные данные'!$B$35:$B$44))</f>
         <v/>
       </c>
       <c r="E35" s="12">
@@ -1745,7 +1752,7 @@
         <v/>
       </c>
       <c r="H35" s="13">
-        <f>IF($A35="","",IF(YEAR($A35)&lt;&gt;YEAR($B35),"Период пересекает 31 декабря — разбейте на две строки",IF($B35&lt;$A35,"Конец периода раньше начала",IF($E35="","Ставка на эту дату не найдена: дополните таблицу ставок",""))))</f>
+        <f>IF($A35="","",IF(YEAR($A35)&lt;&gt;YEAR($B35),"Период пересекает 31 декабря — разбейте на две строки",IF($B35&lt;$A35,"Конец периода раньше начала",IF(OR($B34="",$A35&lt;&gt;$B34+1),"Период пропущен или перекрыт — исправьте даты",IF($E35="","Ставка на эту дату не найдена: дополните таблицу ставок","")))))</f>
         <v/>
       </c>
     </row>
@@ -1757,7 +1764,7 @@
         <v/>
       </c>
       <c r="D36" s="11">
-        <f>IF($A36="","",'Входные данные'!$B$4-SUMIF('Входные данные'!$A$35:$A$44,"&lt;="&amp;$A36,'Входные данные'!$B$35:$B$44))</f>
+        <f>IF($A36="","",'Входные данные'!$B$4-SUMIF('Входные данные'!$A$35:$A$44,"&lt;"&amp;$A36,'Входные данные'!$B$35:$B$44))</f>
         <v/>
       </c>
       <c r="E36" s="12">
@@ -1773,7 +1780,7 @@
         <v/>
       </c>
       <c r="H36" s="13">
-        <f>IF($A36="","",IF(YEAR($A36)&lt;&gt;YEAR($B36),"Период пересекает 31 декабря — разбейте на две строки",IF($B36&lt;$A36,"Конец периода раньше начала",IF($E36="","Ставка на эту дату не найдена: дополните таблицу ставок",""))))</f>
+        <f>IF($A36="","",IF(YEAR($A36)&lt;&gt;YEAR($B36),"Период пересекает 31 декабря — разбейте на две строки",IF($B36&lt;$A36,"Конец периода раньше начала",IF(OR($B35="",$A36&lt;&gt;$B35+1),"Период пропущен или перекрыт — исправьте даты",IF($E36="","Ставка на эту дату не найдена: дополните таблицу ставок","")))))</f>
         <v/>
       </c>
     </row>
@@ -1785,7 +1792,7 @@
         <v/>
       </c>
       <c r="D37" s="11">
-        <f>IF($A37="","",'Входные данные'!$B$4-SUMIF('Входные данные'!$A$35:$A$44,"&lt;="&amp;$A37,'Входные данные'!$B$35:$B$44))</f>
+        <f>IF($A37="","",'Входные данные'!$B$4-SUMIF('Входные данные'!$A$35:$A$44,"&lt;"&amp;$A37,'Входные данные'!$B$35:$B$44))</f>
         <v/>
       </c>
       <c r="E37" s="12">
@@ -1801,7 +1808,7 @@
         <v/>
       </c>
       <c r="H37" s="13">
-        <f>IF($A37="","",IF(YEAR($A37)&lt;&gt;YEAR($B37),"Период пересекает 31 декабря — разбейте на две строки",IF($B37&lt;$A37,"Конец периода раньше начала",IF($E37="","Ставка на эту дату не найдена: дополните таблицу ставок",""))))</f>
+        <f>IF($A37="","",IF(YEAR($A37)&lt;&gt;YEAR($B37),"Период пересекает 31 декабря — разбейте на две строки",IF($B37&lt;$A37,"Конец периода раньше начала",IF(OR($B36="",$A37&lt;&gt;$B36+1),"Период пропущен или перекрыт — исправьте даты",IF($E37="","Ставка на эту дату не найдена: дополните таблицу ставок","")))))</f>
         <v/>
       </c>
     </row>
@@ -1813,7 +1820,7 @@
         <v/>
       </c>
       <c r="D38" s="11">
-        <f>IF($A38="","",'Входные данные'!$B$4-SUMIF('Входные данные'!$A$35:$A$44,"&lt;="&amp;$A38,'Входные данные'!$B$35:$B$44))</f>
+        <f>IF($A38="","",'Входные данные'!$B$4-SUMIF('Входные данные'!$A$35:$A$44,"&lt;"&amp;$A38,'Входные данные'!$B$35:$B$44))</f>
         <v/>
       </c>
       <c r="E38" s="12">
@@ -1829,7 +1836,7 @@
         <v/>
       </c>
       <c r="H38" s="13">
-        <f>IF($A38="","",IF(YEAR($A38)&lt;&gt;YEAR($B38),"Период пересекает 31 декабря — разбейте на две строки",IF($B38&lt;$A38,"Конец периода раньше начала",IF($E38="","Ставка на эту дату не найдена: дополните таблицу ставок",""))))</f>
+        <f>IF($A38="","",IF(YEAR($A38)&lt;&gt;YEAR($B38),"Период пересекает 31 декабря — разбейте на две строки",IF($B38&lt;$A38,"Конец периода раньше начала",IF(OR($B37="",$A38&lt;&gt;$B37+1),"Период пропущен или перекрыт — исправьте даты",IF($E38="","Ставка на эту дату не найдена: дополните таблицу ставок","")))))</f>
         <v/>
       </c>
     </row>
@@ -1841,7 +1848,7 @@
         <v/>
       </c>
       <c r="D39" s="11">
-        <f>IF($A39="","",'Входные данные'!$B$4-SUMIF('Входные данные'!$A$35:$A$44,"&lt;="&amp;$A39,'Входные данные'!$B$35:$B$44))</f>
+        <f>IF($A39="","",'Входные данные'!$B$4-SUMIF('Входные данные'!$A$35:$A$44,"&lt;"&amp;$A39,'Входные данные'!$B$35:$B$44))</f>
         <v/>
       </c>
       <c r="E39" s="12">
@@ -1857,7 +1864,7 @@
         <v/>
       </c>
       <c r="H39" s="13">
-        <f>IF($A39="","",IF(YEAR($A39)&lt;&gt;YEAR($B39),"Период пересекает 31 декабря — разбейте на две строки",IF($B39&lt;$A39,"Конец периода раньше начала",IF($E39="","Ставка на эту дату не найдена: дополните таблицу ставок",""))))</f>
+        <f>IF($A39="","",IF(YEAR($A39)&lt;&gt;YEAR($B39),"Период пересекает 31 декабря — разбейте на две строки",IF($B39&lt;$A39,"Конец периода раньше начала",IF(OR($B38="",$A39&lt;&gt;$B38+1),"Период пропущен или перекрыт — исправьте даты",IF($E39="","Ставка на эту дату не найдена: дополните таблицу ставок","")))))</f>
         <v/>
       </c>
     </row>
@@ -1869,7 +1876,7 @@
         <v/>
       </c>
       <c r="D40" s="11">
-        <f>IF($A40="","",'Входные данные'!$B$4-SUMIF('Входные данные'!$A$35:$A$44,"&lt;="&amp;$A40,'Входные данные'!$B$35:$B$44))</f>
+        <f>IF($A40="","",'Входные данные'!$B$4-SUMIF('Входные данные'!$A$35:$A$44,"&lt;"&amp;$A40,'Входные данные'!$B$35:$B$44))</f>
         <v/>
       </c>
       <c r="E40" s="12">
@@ -1885,7 +1892,7 @@
         <v/>
       </c>
       <c r="H40" s="13">
-        <f>IF($A40="","",IF(YEAR($A40)&lt;&gt;YEAR($B40),"Период пересекает 31 декабря — разбейте на две строки",IF($B40&lt;$A40,"Конец периода раньше начала",IF($E40="","Ставка на эту дату не найдена: дополните таблицу ставок",""))))</f>
+        <f>IF($A40="","",IF(YEAR($A40)&lt;&gt;YEAR($B40),"Период пересекает 31 декабря — разбейте на две строки",IF($B40&lt;$A40,"Конец периода раньше начала",IF(OR($B39="",$A40&lt;&gt;$B39+1),"Период пропущен или перекрыт — исправьте даты",IF($E40="","Ставка на эту дату не найдена: дополните таблицу ставок","")))))</f>
         <v/>
       </c>
     </row>
@@ -1897,7 +1904,7 @@
         <v/>
       </c>
       <c r="D41" s="11">
-        <f>IF($A41="","",'Входные данные'!$B$4-SUMIF('Входные данные'!$A$35:$A$44,"&lt;="&amp;$A41,'Входные данные'!$B$35:$B$44))</f>
+        <f>IF($A41="","",'Входные данные'!$B$4-SUMIF('Входные данные'!$A$35:$A$44,"&lt;"&amp;$A41,'Входные данные'!$B$35:$B$44))</f>
         <v/>
       </c>
       <c r="E41" s="12">
@@ -1913,7 +1920,7 @@
         <v/>
       </c>
       <c r="H41" s="13">
-        <f>IF($A41="","",IF(YEAR($A41)&lt;&gt;YEAR($B41),"Период пересекает 31 декабря — разбейте на две строки",IF($B41&lt;$A41,"Конец периода раньше начала",IF($E41="","Ставка на эту дату не найдена: дополните таблицу ставок",""))))</f>
+        <f>IF($A41="","",IF(YEAR($A41)&lt;&gt;YEAR($B41),"Период пересекает 31 декабря — разбейте на две строки",IF($B41&lt;$A41,"Конец периода раньше начала",IF(OR($B40="",$A41&lt;&gt;$B40+1),"Период пропущен или перекрыт — исправьте даты",IF($E41="","Ставка на эту дату не найдена: дополните таблицу ставок","")))))</f>
         <v/>
       </c>
     </row>
@@ -1925,7 +1932,7 @@
         <v/>
       </c>
       <c r="D42" s="11">
-        <f>IF($A42="","",'Входные данные'!$B$4-SUMIF('Входные данные'!$A$35:$A$44,"&lt;="&amp;$A42,'Входные данные'!$B$35:$B$44))</f>
+        <f>IF($A42="","",'Входные данные'!$B$4-SUMIF('Входные данные'!$A$35:$A$44,"&lt;"&amp;$A42,'Входные данные'!$B$35:$B$44))</f>
         <v/>
       </c>
       <c r="E42" s="12">
@@ -1941,7 +1948,7 @@
         <v/>
       </c>
       <c r="H42" s="13">
-        <f>IF($A42="","",IF(YEAR($A42)&lt;&gt;YEAR($B42),"Период пересекает 31 декабря — разбейте на две строки",IF($B42&lt;$A42,"Конец периода раньше начала",IF($E42="","Ставка на эту дату не найдена: дополните таблицу ставок",""))))</f>
+        <f>IF($A42="","",IF(YEAR($A42)&lt;&gt;YEAR($B42),"Период пересекает 31 декабря — разбейте на две строки",IF($B42&lt;$A42,"Конец периода раньше начала",IF(OR($B41="",$A42&lt;&gt;$B41+1),"Период пропущен или перекрыт — исправьте даты",IF($E42="","Ставка на эту дату не найдена: дополните таблицу ставок","")))))</f>
         <v/>
       </c>
     </row>
@@ -1953,7 +1960,7 @@
         <v/>
       </c>
       <c r="D43" s="11">
-        <f>IF($A43="","",'Входные данные'!$B$4-SUMIF('Входные данные'!$A$35:$A$44,"&lt;="&amp;$A43,'Входные данные'!$B$35:$B$44))</f>
+        <f>IF($A43="","",'Входные данные'!$B$4-SUMIF('Входные данные'!$A$35:$A$44,"&lt;"&amp;$A43,'Входные данные'!$B$35:$B$44))</f>
         <v/>
       </c>
       <c r="E43" s="12">
@@ -1969,7 +1976,7 @@
         <v/>
       </c>
       <c r="H43" s="13">
-        <f>IF($A43="","",IF(YEAR($A43)&lt;&gt;YEAR($B43),"Период пересекает 31 декабря — разбейте на две строки",IF($B43&lt;$A43,"Конец периода раньше начала",IF($E43="","Ставка на эту дату не найдена: дополните таблицу ставок",""))))</f>
+        <f>IF($A43="","",IF(YEAR($A43)&lt;&gt;YEAR($B43),"Период пересекает 31 декабря — разбейте на две строки",IF($B43&lt;$A43,"Конец периода раньше начала",IF(OR($B42="",$A43&lt;&gt;$B42+1),"Период пропущен или перекрыт — исправьте даты",IF($E43="","Ставка на эту дату не найдена: дополните таблицу ставок","")))))</f>
         <v/>
       </c>
     </row>
@@ -1981,6 +1988,10 @@
       </c>
       <c r="G45" s="15">
         <f>ROUND(SUM($G$4:$G$43),2)</f>
+        <v/>
+      </c>
+      <c r="H45" s="16">
+        <f>IF(COUNT($A$4:$A$43)=0,"",IF(MAX($B$4:$B$43)&lt;&gt;'Входные данные'!$B$6,"Последний период не совпадает с датой окончания",""))</f>
         <v/>
       </c>
     </row>
@@ -2053,89 +2064,89 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="16" t="inlineStr">
+      <c r="A4" s="17" t="inlineStr">
         <is>
           <t>Сумма долга на начало расчёта, руб.</t>
         </is>
       </c>
-      <c r="B4" s="17">
+      <c r="B4" s="18">
         <f>'Входные данные'!$B$4</f>
         <v/>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="16" t="inlineStr">
+      <c r="A5" s="17" t="inlineStr">
         <is>
           <t>Учтено частичных оплат, руб.</t>
         </is>
       </c>
-      <c r="B5" s="17">
+      <c r="B5" s="18">
         <f>ROUND(SUM('Входные данные'!$B$35:$B$44),2)</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="16" t="inlineStr">
+      <c r="A6" s="17" t="inlineStr">
         <is>
           <t>Основной долг к взысканию, руб.</t>
         </is>
       </c>
-      <c r="B6" s="17">
+      <c r="B6" s="18">
         <f>ROUND('Входные данные'!$B$4-SUM('Входные данные'!$B$35:$B$44),2)</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="16" t="inlineStr">
+      <c r="A7" s="17" t="inlineStr">
         <is>
           <t>Период начисления с</t>
         </is>
       </c>
-      <c r="B7" s="18">
+      <c r="B7" s="19">
         <f>'Входные данные'!$B$5</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="16" t="inlineStr">
+      <c r="A8" s="17" t="inlineStr">
         <is>
           <t>Период начисления по</t>
         </is>
       </c>
-      <c r="B8" s="18">
+      <c r="B8" s="19">
         <f>'Входные данные'!$B$6</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="16" t="inlineStr">
+      <c r="A9" s="17" t="inlineStr">
         <is>
           <t>Всего дней просрочки</t>
         </is>
       </c>
-      <c r="B9" s="19">
+      <c r="B9" s="20">
         <f>IF(OR('Входные данные'!$B$5="",'Входные данные'!$B$6=""),"",'Входные данные'!$B$6-'Входные данные'!$B$5+1)</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="16" t="inlineStr">
+      <c r="A10" s="17" t="inlineStr">
         <is>
           <t>Проценты по ст. 395 ГК РФ, руб.</t>
         </is>
       </c>
-      <c r="B10" s="17">
+      <c r="B10" s="18">
         <f>'Расчёт'!$G$45</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="16" t="inlineStr">
+      <c r="A11" s="17" t="inlineStr">
         <is>
           <t>Итого к взысканию, руб.</t>
         </is>
       </c>
-      <c r="B11" s="17">
+      <c r="B11" s="18">
         <f>'Расчёт'!$G$46</f>
         <v/>
       </c>
@@ -2148,7 +2159,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="20" t="inlineStr">
+      <c r="A13" s="21" t="inlineStr">
         <is>
           <t>Проценты подлежат начислению по день фактической уплаты долга (п. 3 ст. 395 ГК РФ).</t>
         </is>
@@ -2228,7 +2239,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="21" t="inlineStr">
+      <c r="A2" s="22" t="inlineStr">
         <is>
           <t>Здесь показан формат ввода, а не ваш расчёт. Цифры вымышленные, ставки — условные: реальные берите на cbr.ru. Ничего отсюда не переносите в документ.</t>
         </is>
@@ -2242,36 +2253,36 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="20" t="inlineStr">
+      <c r="A5" s="21" t="inlineStr">
         <is>
           <t>Сумма долга, руб.</t>
         </is>
       </c>
-      <c r="B5" s="22" t="inlineStr">
+      <c r="B5" s="23" t="inlineStr">
         <is>
           <t>1 250 000,00</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="20" t="inlineStr">
+      <c r="A6" s="21" t="inlineStr">
         <is>
           <t>Дата начала просрочки</t>
         </is>
       </c>
-      <c r="B6" s="22" t="inlineStr">
+      <c r="B6" s="23" t="inlineStr">
         <is>
           <t>15.03.2026</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="20" t="inlineStr">
+      <c r="A7" s="21" t="inlineStr">
         <is>
           <t>Дата окончания расчёта</t>
         </is>
       </c>
-      <c r="B7" s="22" t="inlineStr">
+      <c r="B7" s="23" t="inlineStr">
         <is>
           <t>30.07.2026</t>
         </is>
@@ -2297,24 +2308,24 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="22" t="inlineStr">
+      <c r="A11" s="23" t="inlineStr">
         <is>
           <t>15.03.2026</t>
         </is>
       </c>
-      <c r="B11" s="22" t="inlineStr">
+      <c r="B11" s="23" t="inlineStr">
         <is>
           <t>условная 1</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="22" t="inlineStr">
+      <c r="A12" s="23" t="inlineStr">
         <is>
           <t>28.04.2026</t>
         </is>
       </c>
-      <c r="B12" s="22" t="inlineStr">
+      <c r="B12" s="23" t="inlineStr">
         <is>
           <t>условная 2</t>
         </is>
@@ -2370,84 +2381,84 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="23" t="inlineStr">
+      <c r="A16" s="24" t="inlineStr">
         <is>
           <t>15.03.2026</t>
         </is>
       </c>
-      <c r="B16" s="23" t="inlineStr">
+      <c r="B16" s="24" t="inlineStr">
         <is>
           <t>27.04.2026</t>
         </is>
       </c>
-      <c r="C16" s="24" t="inlineStr">
+      <c r="C16" s="25" t="inlineStr">
         <is>
           <t>считается</t>
         </is>
       </c>
-      <c r="D16" s="24" t="inlineStr">
+      <c r="D16" s="25" t="inlineStr">
         <is>
           <t>считается</t>
         </is>
       </c>
-      <c r="E16" s="24" t="inlineStr">
+      <c r="E16" s="25" t="inlineStr">
         <is>
           <t>подставится</t>
         </is>
       </c>
-      <c r="F16" s="24" t="inlineStr">
+      <c r="F16" s="25" t="inlineStr">
         <is>
           <t>считается</t>
         </is>
       </c>
-      <c r="G16" s="24" t="inlineStr">
+      <c r="G16" s="25" t="inlineStr">
         <is>
           <t>считается</t>
         </is>
       </c>
-      <c r="H16" s="24" t="inlineStr">
+      <c r="H16" s="25" t="inlineStr">
         <is>
           <t>пусто, если всё верно</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="23" t="inlineStr">
+      <c r="A17" s="24" t="inlineStr">
         <is>
           <t>28.04.2026</t>
         </is>
       </c>
-      <c r="B17" s="23" t="inlineStr">
+      <c r="B17" s="24" t="inlineStr">
         <is>
           <t>30.07.2026</t>
         </is>
       </c>
-      <c r="C17" s="24" t="inlineStr">
+      <c r="C17" s="25" t="inlineStr">
         <is>
           <t>считается</t>
         </is>
       </c>
-      <c r="D17" s="24" t="inlineStr">
+      <c r="D17" s="25" t="inlineStr">
         <is>
           <t>считается</t>
         </is>
       </c>
-      <c r="E17" s="24" t="inlineStr">
+      <c r="E17" s="25" t="inlineStr">
         <is>
           <t>подставится</t>
         </is>
       </c>
-      <c r="F17" s="24" t="inlineStr">
+      <c r="F17" s="25" t="inlineStr">
         <is>
           <t>считается</t>
         </is>
       </c>
-      <c r="G17" s="24" t="inlineStr">
+      <c r="G17" s="25" t="inlineStr">
         <is>
           <t>считается</t>
         </is>
       </c>
-      <c r="H17" s="24" t="inlineStr">
+      <c r="H17" s="25" t="inlineStr">
         <is>
           <t>пусто, если всё верно</t>
         </is>

</xml_diff>

<commit_message>
fix(p1): deliver independently checked comparison instructions
</commit_message>
<xml_diff>
--- a/products-storage/01-zakrytie-rabot/14-raschet-procentov-395-gk.xlsx
+++ b/products-storage/01-zakrytie-rabot/14-raschet-procentov-395-gk.xlsx
@@ -2026,7 +2026,7 @@
     <row r="51" ht="46" customHeight="1">
       <c r="A51" s="5" t="inlineStr">
         <is>
-          <t>Сверьте итог с любым публичным калькулятором процентов по ст. 395 ГК РФ — например, в справочно-правовой системе. Расхождение больше копеек на округлении означает ошибку в разбивке периодов, а не в калькуляторе. Колонка «Проверка» должна быть пустой во всех заполненных строках.</t>
+          <t>Сверьте итог с независимым расчётом процентов по ст. 395 ГК РФ, например в справочно-правовой системе. При расхождении проверьте ставки, даты, базу долга, разбивку периодов и округление в обоих расчётах. Колонка «Проверка» должна быть пустой во всех заполненных строках.</t>
         </is>
       </c>
     </row>
@@ -2200,7 +2200,7 @@
     <row r="19" ht="46" customHeight="1">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>— Юридическую консультацию и вычитку юристом. Порядок расчёта сверен с текстом действующих норм 16.08.2026: нормативная сверка сопоставляет формулировки и порядок со статьями закона и правовой позиции по вашему спору не оценивает.</t>
+          <t>— Юридическую консультацию и вычитку юристом. Нормативная сверка сопоставляет формулировки и порядок со статьями закона и не заменяет проверку обстоятельств вашего спора.</t>
         </is>
       </c>
     </row>

</xml_diff>